<commit_message>
Release v6.14.3 – Financial Analysis import validation improvements
- Updated Financial Analysis Tool to v1.8.1
- Fixed import validation for optional Budget and Forecast sheets
- Changed partial Cost Center allocations from blocking errors to warnings
- Improved import diagnostics and user feedback
- Updated related website pages and templates
</commit_message>
<xml_diff>
--- a/resources/templates/Template_Analisi_di_Bilancio_AI.xlsx
+++ b/resources/templates/Template_Analisi_di_Bilancio_AI.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="R0135cca852404be0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="Rc7ed845f95ca4e36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voci IV Direttiva" sheetId="3" r:id="Rce90814551ba44e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stato Patrimoniale" sheetId="4" r:id="R02458731ee0142be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conto Economico" sheetId="5" r:id="Re0bb187d17ca42fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Esiti AI" sheetId="6" r:id="R45a4f5c0d5af4238"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="7" r:id="R1daf76df4ceb4715"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="8" r:id="R08c04d9b5e3146c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo centri" sheetId="9" r:id="Rf7ebb865bc75494a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocazioni centri" sheetId="10" r:id="R5c840f323daa49af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="R8ebde0d11c5c44c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="Re6795b487f5b48eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voci IV Direttiva" sheetId="3" r:id="R396872b388ad4a90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stato Patrimoniale" sheetId="4" r:id="R8c7578a55df34e38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conto Economico" sheetId="5" r:id="Rd76256e884c44303"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Esiti AI" sheetId="6" r:id="Rc8c827a1f3424790"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="7" r:id="Ra02039a41a0747d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="8" r:id="R8a42675ba7f04fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo centri" sheetId="9" r:id="R61f875da84e74b07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocazioni centri" sheetId="10" r:id="R1ebabeae6c914ca7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -340,12 +340,12 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="2" t="str">
-        <x:v>Budget e Forecast: compilare soltanto se disponibili e con valori cumulati alla stessa data e sullo stesso perimetro dell’actual.</x:v>
+        <x:v>Budget e Forecast: inserire soltanto conti del Conto Economico. Le righe di Stato Patrimoniale vengono escluse dal confronto; una copertura parziale è accettata e segnalata come provvisoria.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="2" t="str">
-        <x:v>Catalogo centri e Allocazioni centri: compilare soltanto se si vuole l’analisi per centro di costo. I fogli facoltativi possono restare vuoti.</x:v>
+        <x:v>Catalogo centri e Allocazioni centri: compilare soltanto per l’analisi per centro di costo. È ammessa una copertura parziale, purché ogni conto inserito sia riconciliato; i conti non allocati restano segnalati come avviso.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">

</xml_diff>

<commit_message>
Release v6.15.4 – Add controlled year-end result reconciliation
- Added pre-closing and post-closing balance detection
- Added controlled A.IX technical result reconstruction
- Preserved all original ERP rows and account granularity
- Allowed supported pre-closing imports with professional confirmation
- Blocked final exports until the technical result is confirmed
- Prevented forced balancing where SP and CE do not reconcile
- Improved numeric Excel parsing in Financial Statement
- Updated Financial Analysis to v2.0.4
- Updated Financial Statement to v1.3.3
- Updated Configura con AI prompts and templates in Italian, English and Spanish
</commit_message>
<xml_diff>
--- a/resources/templates/Template_Analisi_di_Bilancio_AI.xlsx
+++ b/resources/templates/Template_Analisi_di_Bilancio_AI.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="Rd6e1f58f14fd4d2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="Raab95d518bbd401f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voci IV Direttiva" sheetId="3" r:id="R94a2203899b842d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stato Patrimoniale" sheetId="4" r:id="R175de554f1a34ce5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conto Economico" sheetId="5" r:id="R0788c37953174741"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Esiti AI" sheetId="6" r:id="R921b0c6904b048f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="7" r:id="Rd173cd364f624f99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="8" r:id="Re5d04a4cad4849d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo centri" sheetId="9" r:id="R717845ff564e4a30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocazioni centri" sheetId="10" r:id="Rb5d36df97df24224"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="R835d16bb29f24893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="R5177964d05014ee8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voci IV Direttiva" sheetId="3" r:id="R7c37c60fce5a4040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stato Patrimoniale" sheetId="4" r:id="Re67e11dc2365490d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conto Economico" sheetId="5" r:id="R152225934bab49c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Esiti AI" sheetId="6" r:id="R4b1a299e8ca14943"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="7" r:id="R1692f570c9c24bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="8" r:id="Rd77939ac80f34c2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo centri" sheetId="9" r:id="R1209c643717a460c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocazioni centri" sheetId="10" r:id="R90e46d1b9ab3446e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1003,7 +1003,7 @@
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="47">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -1120,6 +1120,30 @@
     </x:xf>
     <x:xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="7">
@@ -1340,7 +1364,7 @@
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0">
       <x:c r="A1" s="20" t="str">
-        <x:v>TAX AUTOMATION LAB — ANALISI DI BILANCIO v2.0.0</x:v>
+        <x:v>TAX AUTOMATION LAB — ANALISI DI BILANCIO v2.0.4</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0">
@@ -1384,7 +1408,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="28" t="str">
-        <x:v>Mantieni ogni conto e sottoconto come riga autonoma. Non aggregare righe che condividono lo stesso codice conto.</x:v>
+        <x:v>Mantieni ogni conto, sottoconto e sottosottoconto come riga autonoma. Non aggregare righe che condividono lo stesso codice conto.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="29.850000381469727" hidden="0">
@@ -1394,12 +1418,12 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0">
       <x:c r="A13" s="28" t="str">
-        <x:v>Il numero di righe restituito deve coincidere con il file sorgente, escluse soltanto righe vuote e righe di totale esplicite.</x:v>
+        <x:v>Il numero delle righe sorgente conservate deve coincidere con il file sorgente, escluse soltanto righe vuote e righe di totale esplicite.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0">
       <x:c r="A14" s="28" t="str">
-        <x:v>Assegna a ogni sottoconto la voce IV Direttiva appropriata. Quando la natura è la stessa, i sottoconti possono condividere la categoria del conto principale.</x:v>
+        <x:v>Assegna a ogni sottoconto la voce IV Direttiva appropriata. Quando la natura è la stessa, i sottoconti possono condividere la categoria del conto principale senza essere aggregati.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0">
@@ -1412,30 +1436,32 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0">
       <x:c r="A17" s="24" t="str">
-        <x:v>PRIMO ESERCIZIO</x:v>
+        <x:v>RISULTATO D’ESERCIZIO E QUADRATURA</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0">
       <x:c r="A18" s="28" t="str">
-        <x:v>Se non esiste un esercizio precedente, lascia vuota la relativa colonna e indica nel foglio “Esiti AI” che si tratta del primo esercizio. Non replicare i valori correnti nel comparativo.</x:v>
+        <x:v>Riconosci se il file è un bilancio ante chiusura, post chiusura oppure uno schema già riclassificato. Calcola separatamente saldo dello Stato Patrimoniale e risultato del Conto Economico.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0">
-      <x:c r="A19" s="28"/>
+      <x:c r="A19" s="28" t="str">
+        <x:v>Se il risultato è già presente nel patrimonio netto in A.IX, non aggiungere o duplicare righe.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0">
       <x:c r="A20" s="24" t="str">
-        <x:v>FOGLI FACOLTATIVI</x:v>
+        <x:v>Se A.IX manca e la differenza dello Stato Patrimoniale coincide esattamente, con segno opposto, con il risultato del Conto Economico, conserva tutte le righe originarie e aggiungi una sola riga tecnica: codice TAL_AIX, descrizione “Utile/Perdita dell’esercizio — voce tecnica derivata”, voce AIX.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0">
       <x:c r="A21" s="28" t="str">
-        <x:v>Budget e Forecast: inserire soltanto conti del Conto Economico. Le righe di Stato Patrimoniale sono escluse dal confronto; una copertura parziale è accettata e segnalata come provvisoria.</x:v>
+        <x:v>La riga TAL_AIX è aggiuntiva e non è un codice ERP. Documentala nel foglio “Esiti AI” indicando saldo SP, risultato CE, importo ricostruito, quadratura finale e verifica richiesta al professionista.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0">
       <x:c r="A22" s="28" t="str">
-        <x:v>Catalogo centri e Allocazioni centri: è ammessa una copertura parziale, purché ogni conto allocato sia riconciliato; i conti non allocati restano segnalati come avviso.</x:v>
+        <x:v>Se la differenza dello Stato Patrimoniale non coincide con il risultato del Conto Economico, non forzare la quadratura e non creare conti compensativi: segnala l’anomalia in “Esiti AI”.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="29.850000381469727" hidden="0">
@@ -1443,34 +1469,65 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="29" t="str">
-        <x:v>REGOLE DI QUALITÀ</x:v>
+        <x:v>PRIMO ESERCIZIO</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="30" t="str">
-        <x:v>Non inventare dati, mapping, benchmark, driver o allocazioni. Inserisci valori, non formule o collegamenti esterni.</x:v>
+        <x:v>Se non esiste un esercizio precedente, lascia vuota la relativa colonna e indica nel foglio “Esiti AI” che si tratta del primo esercizio. Non replicare i valori correnti nel comparativo.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="30" t="str">
-        <x:v>Non eliminare fogli, non cambiare le intestazioni e non aggiungere colonne ai fogli importati dal tool.</x:v>
-      </x:c>
+      <x:c r="A26" s="30"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="30" t="str">
-        <x:v>Documenta nel foglio “Esiti AI” fonti, assunzioni, dubbi e verifiche richieste al professionista.</x:v>
+        <x:v>FOGLI FACOLTATIVI</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="30"/>
+      <x:c r="A28" s="30" t="str">
+        <x:v>Budget e Forecast: inserire soltanto conti del Conto Economico. Le righe di Stato Patrimoniale sono escluse dal confronto; una copertura parziale è accettata e segnalata come provvisoria.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="29" t="str">
+        <x:v>Catalogo centri e Allocazioni centri: è ammessa una copertura parziale, purché ogni conto allocato sia riconciliato; i conti non allocati restano segnalati come avviso.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="30" t="str">
+        <x:v>REGOLE DI QUALITÀ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="30" t="str">
+        <x:v>Non inventare dati, mapping, benchmark, driver o allocazioni. Inserisci valori, non formule o collegamenti esterni.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="30" t="str">
+        <x:v>Non eliminare fogli, non cambiare le intestazioni e non aggiungere colonne ai fogli importati dal tool.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="30" t="str">
+        <x:v>Documenta nel foglio “Esiti AI” fonti, assunzioni, tipo di bilancio rilevato, convenzione dei segni, eventuali righe tecniche, dubbi e verifiche richieste al professionista.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="30"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="30" t="str">
         <x:v>VERIFICA PROFESSIONALE</x:v>
       </x:c>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="30" t="str">
+    <x:row r="37">
+      <x:c r="A37" s="30" t="str">
         <x:v>Il file deve essere controllato dal professionista prima dell’importazione. L’AI assiste la preparazione tecnica ma non sostituisce la valutazione contabile e finanziaria.</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Release v6.15.8 – Harden XLSX exports and fix Financial Analysis downloads
</commit_message>
<xml_diff>
--- a/resources/templates/Template_Analisi_di_Bilancio_AI.xlsx
+++ b/resources/templates/Template_Analisi_di_Bilancio_AI.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="R835d16bb29f24893"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="R5177964d05014ee8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voci IV Direttiva" sheetId="3" r:id="R7c37c60fce5a4040"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stato Patrimoniale" sheetId="4" r:id="Re67e11dc2365490d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conto Economico" sheetId="5" r:id="R152225934bab49c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Esiti AI" sheetId="6" r:id="R4b1a299e8ca14943"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="7" r:id="R1692f570c9c24bb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="8" r:id="Rd77939ac80f34c2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo centri" sheetId="9" r:id="R1209c643717a460c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocazioni centri" sheetId="10" r:id="R90e46d1b9ab3446e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="Ree183eed13144f0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="R7614d7a6e9e64a47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voci IV Direttiva" sheetId="3" r:id="Rf45c523a5b7c4bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stato Patrimoniale" sheetId="4" r:id="Ra45b3708c75f4c46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conto Economico" sheetId="5" r:id="Rcf2fce5651dd44f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Esiti AI" sheetId="6" r:id="R5b549bf3897c45ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="7" r:id="R375e262a06a046f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="8" r:id="R2f179c2e59f54645"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo centri" sheetId="9" r:id="R77cc9196a5af4ef6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocazioni centri" sheetId="10" r:id="R6a6824b53e954657"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1261,9 +1261,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1364,7 +1364,7 @@
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0">
       <x:c r="A1" s="20" t="str">
-        <x:v>TAX AUTOMATION LAB — ANALISI DI BILANCIO v2.0.4</x:v>
+        <x:v>TAX AUTOMATION LAB — ANALISI DI BILANCIO v2.0.6</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0">

</xml_diff>